<commit_message>
Fixed mistake in supplementary file for Sigma Aldrich Equine IGFBP2 on contributor request
</commit_message>
<xml_diff>
--- a/_data/supplementary/344a9db6870ae81a03ffa2706_Sigma_Aldrich_Equine_IGFBP2_ELISA/Equine_IGFBP2_Sigma_07_30_26.xlsx
+++ b/_data/supplementary/344a9db6870ae81a03ffa2706_Sigma_Aldrich_Equine_IGFBP2_ELISA/Equine_IGFBP2_Sigma_07_30_26.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mstate-my.sharepoint.com/personal/ma2020_msstate_edu/Documents/Documents 1/ELISA Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jrd699\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="13_ncr:1_{A8A128DB-46EE-41BF-ACD8-2AD24CA4CB62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C28B7BC-F646-467B-864D-3FE26566E20B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31E231DA-7AAC-4611-8C7C-7C755CD1CD70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-13410" yWindow="-24120" windowWidth="57840" windowHeight="23520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Absorbance 1_01" sheetId="1" r:id="rId1"/>
@@ -878,7 +878,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -933,14 +933,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -953,18 +946,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1821,7 +1818,7 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="39" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="14" t="s">
@@ -1836,17 +1833,17 @@
       <c r="E5" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="31"/>
-      <c r="M5" s="31"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
+      <c r="K5" s="40"/>
+      <c r="L5" s="40"/>
+      <c r="M5" s="40"/>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="31"/>
+      <c r="A6" s="40"/>
       <c r="B6" s="16" t="s">
         <v>187</v>
       </c>
@@ -1859,17 +1856,17 @@
       <c r="E6" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
-      <c r="K6" s="31"/>
-      <c r="L6" s="31"/>
-      <c r="M6" s="31"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="40"/>
+      <c r="K6" s="40"/>
+      <c r="L6" s="40"/>
+      <c r="M6" s="40"/>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="31"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="18" t="s">
         <v>188</v>
       </c>
@@ -1882,17 +1879,17 @@
       <c r="E7" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="F7" s="31"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="31"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="31"/>
-      <c r="L7" s="31"/>
-      <c r="M7" s="31"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="40"/>
+      <c r="H7" s="40"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="40"/>
+      <c r="L7" s="40"/>
+      <c r="M7" s="40"/>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="39" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="14" t="s">
@@ -1907,17 +1904,17 @@
       <c r="E8" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="31"/>
-      <c r="L8" s="31"/>
-      <c r="M8" s="31"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="40"/>
+      <c r="K8" s="40"/>
+      <c r="L8" s="40"/>
+      <c r="M8" s="40"/>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="31"/>
+      <c r="A9" s="40"/>
       <c r="B9" s="16" t="s">
         <v>187</v>
       </c>
@@ -1930,17 +1927,17 @@
       <c r="E9" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31"/>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
+      <c r="F9" s="40"/>
+      <c r="G9" s="40"/>
+      <c r="H9" s="40"/>
+      <c r="I9" s="40"/>
+      <c r="J9" s="40"/>
+      <c r="K9" s="40"/>
+      <c r="L9" s="40"/>
+      <c r="M9" s="40"/>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="31"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="18" t="s">
         <v>190</v>
       </c>
@@ -1953,17 +1950,17 @@
       <c r="E10" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="31"/>
-      <c r="K10" s="31"/>
-      <c r="L10" s="31"/>
-      <c r="M10" s="31"/>
+      <c r="F10" s="40"/>
+      <c r="G10" s="40"/>
+      <c r="H10" s="40"/>
+      <c r="I10" s="40"/>
+      <c r="J10" s="40"/>
+      <c r="K10" s="40"/>
+      <c r="L10" s="40"/>
+      <c r="M10" s="40"/>
     </row>
     <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="39" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="14" t="s">
@@ -1978,17 +1975,17 @@
       <c r="E11" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="31"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="31"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="31"/>
-      <c r="L11" s="31"/>
-      <c r="M11" s="31"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
+      <c r="K11" s="40"/>
+      <c r="L11" s="40"/>
+      <c r="M11" s="40"/>
     </row>
     <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="31"/>
+      <c r="A12" s="40"/>
       <c r="B12" s="16" t="s">
         <v>187</v>
       </c>
@@ -2001,17 +1998,17 @@
       <c r="E12" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="F12" s="31"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="31"/>
-      <c r="I12" s="31"/>
-      <c r="J12" s="31"/>
-      <c r="K12" s="31"/>
-      <c r="L12" s="31"/>
-      <c r="M12" s="31"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="40"/>
+      <c r="K12" s="40"/>
+      <c r="L12" s="40"/>
+      <c r="M12" s="40"/>
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="31"/>
+      <c r="A13" s="40"/>
       <c r="B13" s="18" t="s">
         <v>191</v>
       </c>
@@ -2024,17 +2021,17 @@
       <c r="E13" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="F13" s="31"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="31"/>
-      <c r="I13" s="31"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="31"/>
-      <c r="L13" s="31"/>
-      <c r="M13" s="31"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="40"/>
+      <c r="J13" s="40"/>
+      <c r="K13" s="40"/>
+      <c r="L13" s="40"/>
+      <c r="M13" s="40"/>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="39" t="s">
         <v>11</v>
       </c>
       <c r="B14" s="14" t="s">
@@ -2049,17 +2046,17 @@
       <c r="E14" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="F14" s="31"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
-      <c r="I14" s="31"/>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="31"/>
-      <c r="M14" s="31"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="40"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="40"/>
+      <c r="J14" s="40"/>
+      <c r="K14" s="40"/>
+      <c r="L14" s="40"/>
+      <c r="M14" s="40"/>
     </row>
     <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="31"/>
+      <c r="A15" s="40"/>
       <c r="B15" s="16" t="s">
         <v>187</v>
       </c>
@@ -2072,17 +2069,17 @@
       <c r="E15" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="31"/>
-      <c r="I15" s="31"/>
-      <c r="J15" s="31"/>
-      <c r="K15" s="31"/>
-      <c r="L15" s="31"/>
-      <c r="M15" s="31"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="40"/>
+      <c r="K15" s="40"/>
+      <c r="L15" s="40"/>
+      <c r="M15" s="40"/>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="31"/>
+      <c r="A16" s="40"/>
       <c r="B16" s="18" t="s">
         <v>192</v>
       </c>
@@ -2095,17 +2092,17 @@
       <c r="E16" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="31"/>
-      <c r="I16" s="31"/>
-      <c r="J16" s="31"/>
-      <c r="K16" s="31"/>
-      <c r="L16" s="31"/>
-      <c r="M16" s="31"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="40"/>
+      <c r="K16" s="40"/>
+      <c r="L16" s="40"/>
+      <c r="M16" s="40"/>
     </row>
     <row r="17" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="39" t="s">
         <v>12</v>
       </c>
       <c r="B17" s="14" t="s">
@@ -2120,17 +2117,17 @@
       <c r="E17" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="F17" s="31"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="31"/>
-      <c r="I17" s="31"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="31"/>
-      <c r="L17" s="31"/>
-      <c r="M17" s="31"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="40"/>
+      <c r="I17" s="40"/>
+      <c r="J17" s="40"/>
+      <c r="K17" s="40"/>
+      <c r="L17" s="40"/>
+      <c r="M17" s="40"/>
     </row>
     <row r="18" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="31"/>
+      <c r="A18" s="40"/>
       <c r="B18" s="16" t="s">
         <v>187</v>
       </c>
@@ -2143,17 +2140,17 @@
       <c r="E18" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="31"/>
-      <c r="I18" s="31"/>
-      <c r="J18" s="31"/>
-      <c r="K18" s="31"/>
-      <c r="L18" s="31"/>
-      <c r="M18" s="31"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="40"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="40"/>
+      <c r="M18" s="40"/>
     </row>
     <row r="19" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="31"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="18" t="s">
         <v>193</v>
       </c>
@@ -2166,17 +2163,17 @@
       <c r="E19" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="31"/>
-      <c r="I19" s="31"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="31"/>
-      <c r="L19" s="31"/>
-      <c r="M19" s="31"/>
+      <c r="F19" s="40"/>
+      <c r="G19" s="40"/>
+      <c r="H19" s="40"/>
+      <c r="I19" s="40"/>
+      <c r="J19" s="40"/>
+      <c r="K19" s="40"/>
+      <c r="L19" s="40"/>
+      <c r="M19" s="40"/>
     </row>
     <row r="20" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="39" t="s">
         <v>13</v>
       </c>
       <c r="B20" s="14" t="s">
@@ -2191,17 +2188,17 @@
       <c r="E20" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="31"/>
-      <c r="M20" s="31"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
+      <c r="I20" s="40"/>
+      <c r="J20" s="40"/>
+      <c r="K20" s="40"/>
+      <c r="L20" s="40"/>
+      <c r="M20" s="40"/>
     </row>
     <row r="21" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="31"/>
+      <c r="A21" s="40"/>
       <c r="B21" s="16" t="s">
         <v>187</v>
       </c>
@@ -2214,17 +2211,17 @@
       <c r="E21" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="F21" s="31"/>
-      <c r="G21" s="31"/>
-      <c r="H21" s="31"/>
-      <c r="I21" s="31"/>
-      <c r="J21" s="31"/>
-      <c r="K21" s="31"/>
-      <c r="L21" s="31"/>
-      <c r="M21" s="31"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="40"/>
+      <c r="K21" s="40"/>
+      <c r="L21" s="40"/>
+      <c r="M21" s="40"/>
     </row>
     <row r="22" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="31"/>
+      <c r="A22" s="40"/>
       <c r="B22" s="18" t="s">
         <v>194</v>
       </c>
@@ -2237,17 +2234,17 @@
       <c r="E22" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="F22" s="31"/>
-      <c r="G22" s="31"/>
-      <c r="H22" s="31"/>
-      <c r="I22" s="31"/>
-      <c r="J22" s="31"/>
-      <c r="K22" s="31"/>
-      <c r="L22" s="31"/>
-      <c r="M22" s="31"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="40"/>
+      <c r="J22" s="40"/>
+      <c r="K22" s="40"/>
+      <c r="L22" s="40"/>
+      <c r="M22" s="40"/>
     </row>
     <row r="23" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="39" t="s">
         <v>14</v>
       </c>
       <c r="B23" s="14" t="s">
@@ -2262,17 +2259,17 @@
       <c r="E23" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="F23" s="31"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="31"/>
-      <c r="I23" s="31"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="31"/>
-      <c r="L23" s="31"/>
-      <c r="M23" s="31"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="40"/>
+      <c r="I23" s="40"/>
+      <c r="J23" s="40"/>
+      <c r="K23" s="40"/>
+      <c r="L23" s="40"/>
+      <c r="M23" s="40"/>
     </row>
     <row r="24" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="31"/>
+      <c r="A24" s="40"/>
       <c r="B24" s="16" t="s">
         <v>187</v>
       </c>
@@ -2285,17 +2282,17 @@
       <c r="E24" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="F24" s="31"/>
-      <c r="G24" s="31"/>
-      <c r="H24" s="31"/>
-      <c r="I24" s="31"/>
-      <c r="J24" s="31"/>
-      <c r="K24" s="31"/>
-      <c r="L24" s="31"/>
-      <c r="M24" s="31"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="40"/>
+      <c r="J24" s="40"/>
+      <c r="K24" s="40"/>
+      <c r="L24" s="40"/>
+      <c r="M24" s="40"/>
     </row>
     <row r="25" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="31"/>
+      <c r="A25" s="40"/>
       <c r="B25" s="18" t="s">
         <v>195</v>
       </c>
@@ -2308,17 +2305,17 @@
       <c r="E25" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="31"/>
-      <c r="J25" s="31"/>
-      <c r="K25" s="31"/>
-      <c r="L25" s="31"/>
-      <c r="M25" s="31"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="40"/>
+      <c r="J25" s="40"/>
+      <c r="K25" s="40"/>
+      <c r="L25" s="40"/>
+      <c r="M25" s="40"/>
     </row>
     <row r="26" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="32" t="s">
+      <c r="A26" s="39" t="s">
         <v>15</v>
       </c>
       <c r="B26" s="20" t="s">
@@ -2333,17 +2330,17 @@
       <c r="E26" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F26" s="31"/>
-      <c r="G26" s="31"/>
-      <c r="H26" s="31"/>
-      <c r="I26" s="31"/>
-      <c r="J26" s="31"/>
-      <c r="K26" s="31"/>
-      <c r="L26" s="31"/>
-      <c r="M26" s="31"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="40"/>
+      <c r="I26" s="40"/>
+      <c r="J26" s="40"/>
+      <c r="K26" s="40"/>
+      <c r="L26" s="40"/>
+      <c r="M26" s="40"/>
     </row>
     <row r="27" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="31"/>
+      <c r="A27" s="40"/>
       <c r="B27" s="21" t="s">
         <v>187</v>
       </c>
@@ -2356,17 +2353,17 @@
       <c r="E27" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="F27" s="31"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="31"/>
-      <c r="I27" s="31"/>
-      <c r="J27" s="31"/>
-      <c r="K27" s="31"/>
-      <c r="L27" s="31"/>
-      <c r="M27" s="31"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="40"/>
+      <c r="I27" s="40"/>
+      <c r="J27" s="40"/>
+      <c r="K27" s="40"/>
+      <c r="L27" s="40"/>
+      <c r="M27" s="40"/>
     </row>
     <row r="28" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="31"/>
+      <c r="A28" s="40"/>
       <c r="B28" s="22"/>
       <c r="C28" s="19" t="s">
         <v>189</v>
@@ -2377,14 +2374,14 @@
       <c r="E28" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="31"/>
-      <c r="I28" s="31"/>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="40"/>
+      <c r="I28" s="40"/>
+      <c r="J28" s="40"/>
+      <c r="K28" s="40"/>
+      <c r="L28" s="40"/>
+      <c r="M28" s="40"/>
     </row>
     <row r="33" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
@@ -2393,6 +2390,62 @@
     </row>
   </sheetData>
   <mergeCells count="72">
+    <mergeCell ref="M20:M22"/>
+    <mergeCell ref="M23:M25"/>
+    <mergeCell ref="M26:M28"/>
+    <mergeCell ref="M5:M7"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="M11:M13"/>
+    <mergeCell ref="M14:M16"/>
+    <mergeCell ref="M17:M19"/>
+    <mergeCell ref="K20:K22"/>
+    <mergeCell ref="K23:K25"/>
+    <mergeCell ref="K26:K28"/>
+    <mergeCell ref="L5:L7"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="L11:L13"/>
+    <mergeCell ref="L14:L16"/>
+    <mergeCell ref="L17:L19"/>
+    <mergeCell ref="L20:L22"/>
+    <mergeCell ref="L23:L25"/>
+    <mergeCell ref="L26:L28"/>
+    <mergeCell ref="K5:K7"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="K11:K13"/>
+    <mergeCell ref="K14:K16"/>
+    <mergeCell ref="K17:K19"/>
+    <mergeCell ref="I20:I22"/>
+    <mergeCell ref="I23:I25"/>
+    <mergeCell ref="I26:I28"/>
+    <mergeCell ref="J5:J7"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="J11:J13"/>
+    <mergeCell ref="J14:J16"/>
+    <mergeCell ref="J17:J19"/>
+    <mergeCell ref="J20:J22"/>
+    <mergeCell ref="J23:J25"/>
+    <mergeCell ref="J26:J28"/>
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="I11:I13"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="I17:I19"/>
+    <mergeCell ref="G20:G22"/>
+    <mergeCell ref="G23:G25"/>
+    <mergeCell ref="G26:G28"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="H20:H22"/>
+    <mergeCell ref="H23:H25"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="G11:G13"/>
+    <mergeCell ref="G14:G16"/>
+    <mergeCell ref="G17:G19"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="A23:A25"/>
     <mergeCell ref="A26:A28"/>
@@ -2409,62 +2462,6 @@
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A14:A16"/>
     <mergeCell ref="A17:A19"/>
-    <mergeCell ref="G20:G22"/>
-    <mergeCell ref="G23:G25"/>
-    <mergeCell ref="G26:G28"/>
-    <mergeCell ref="H5:H7"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="H11:H13"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="H17:H19"/>
-    <mergeCell ref="H20:H22"/>
-    <mergeCell ref="H23:H25"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="G5:G7"/>
-    <mergeCell ref="G8:G10"/>
-    <mergeCell ref="G11:G13"/>
-    <mergeCell ref="G14:G16"/>
-    <mergeCell ref="G17:G19"/>
-    <mergeCell ref="I20:I22"/>
-    <mergeCell ref="I23:I25"/>
-    <mergeCell ref="I26:I28"/>
-    <mergeCell ref="J5:J7"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="J11:J13"/>
-    <mergeCell ref="J14:J16"/>
-    <mergeCell ref="J17:J19"/>
-    <mergeCell ref="J20:J22"/>
-    <mergeCell ref="J23:J25"/>
-    <mergeCell ref="J26:J28"/>
-    <mergeCell ref="I5:I7"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="I11:I13"/>
-    <mergeCell ref="I14:I16"/>
-    <mergeCell ref="I17:I19"/>
-    <mergeCell ref="K20:K22"/>
-    <mergeCell ref="K23:K25"/>
-    <mergeCell ref="K26:K28"/>
-    <mergeCell ref="L5:L7"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="L11:L13"/>
-    <mergeCell ref="L14:L16"/>
-    <mergeCell ref="L17:L19"/>
-    <mergeCell ref="L20:L22"/>
-    <mergeCell ref="L23:L25"/>
-    <mergeCell ref="L26:L28"/>
-    <mergeCell ref="K5:K7"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="K11:K13"/>
-    <mergeCell ref="K14:K16"/>
-    <mergeCell ref="K17:K19"/>
-    <mergeCell ref="M20:M22"/>
-    <mergeCell ref="M23:M25"/>
-    <mergeCell ref="M26:M28"/>
-    <mergeCell ref="M5:M7"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="M11:M13"/>
-    <mergeCell ref="M14:M16"/>
-    <mergeCell ref="M17:M19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3762,7 +3759,7 @@
       <c r="A21" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="34">
+      <c r="B21" s="31">
         <v>0</v>
       </c>
       <c r="C21" s="27">
@@ -4699,11 +4696,11 @@
       </c>
     </row>
     <row r="81" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="I81" s="39" t="s">
+      <c r="I81" s="35" t="s">
         <v>227</v>
       </c>
-      <c r="J81" s="39"/>
-      <c r="K81" s="39"/>
+      <c r="J81" s="35"/>
+      <c r="K81" s="35"/>
     </row>
     <row r="82" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A82" s="23" t="s">
@@ -4768,7 +4765,7 @@
         <v>97.612343258377948</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A84" s="23" t="s">
         <v>9</v>
       </c>
@@ -4913,7 +4910,7 @@
         <v>5.2600699999999998</v>
       </c>
       <c r="F88" s="7"/>
-      <c r="L88" s="33"/>
+      <c r="L88" s="30"/>
     </row>
     <row r="89" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A89" s="23" t="s">
@@ -4966,8 +4963,8 @@
       </c>
       <c r="F92" s="1"/>
       <c r="G92" s="1"/>
-      <c r="I92" s="37"/>
-      <c r="J92" s="35"/>
+      <c r="I92" s="34"/>
+      <c r="J92" s="32"/>
     </row>
     <row r="93" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A93" s="23" t="s">
@@ -4985,10 +4982,10 @@
       <c r="E93" s="23" t="s">
         <v>204</v>
       </c>
-      <c r="I93" s="39" t="s">
+      <c r="I93" s="35" t="s">
         <v>226</v>
       </c>
-      <c r="J93" s="39"/>
+      <c r="J93" s="35"/>
     </row>
     <row r="94" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A94" s="23" t="s">
@@ -5170,12 +5167,12 @@
       <c r="E100" s="23" t="s">
         <v>211</v>
       </c>
-      <c r="I100" s="41" t="s">
+      <c r="I100" s="37" t="s">
         <v>222</v>
       </c>
-      <c r="J100" s="41"/>
-      <c r="K100" s="41"/>
-      <c r="L100" s="40" t="s">
+      <c r="J100" s="37"/>
+      <c r="K100" s="37"/>
+      <c r="L100" s="38" t="s">
         <v>225</v>
       </c>
       <c r="M100" s="38"/>
@@ -5186,11 +5183,11 @@
     </row>
     <row r="101" spans="1:17" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="I101" s="23"/>
-      <c r="J101" s="36" t="s">
+      <c r="J101" s="33" t="s">
+        <v>223</v>
+      </c>
+      <c r="K101" s="33" t="s">
         <v>224</v>
-      </c>
-      <c r="K101" s="36" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="102" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
@@ -5241,10 +5238,10 @@
       </c>
     </row>
     <row r="109" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I109" s="30"/>
-      <c r="J109" s="30"/>
-      <c r="K109" s="30"/>
-      <c r="L109" s="30"/>
+      <c r="I109" s="36"/>
+      <c r="J109" s="36"/>
+      <c r="K109" s="36"/>
+      <c r="L109" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>